<commit_message>
Add Excel validation workflow and apartment validator
</commit_message>
<xml_diff>
--- a/Central_NJ_Apartment_Comparison_WITH_TOUR_CLUSTERS_FINAL.xlsx
+++ b/Central_NJ_Apartment_Comparison_WITH_TOUR_CLUSTERS_FINAL.xlsx
@@ -545,8 +545,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:S55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -659,6 +659,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -743,6 +748,11 @@
         </is>
       </c>
       <c r="R2" s="4" t="str"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -831,6 +841,11 @@
           <t>https://www.apartments.com/fairway-28-bridgewater-nj/3m3bv0f/</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -919,6 +934,11 @@
           <t>https://www.apartments.com/station-house-somerville-nj/0bzvy20/</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1007,6 +1027,11 @@
           <t>https://www.queensgateapts.com/floorplans</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1095,6 +1120,11 @@
           <t>https://www.redfin.com/zipcode/08854/2-bedroom-houses-for-rent</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1183,6 +1213,11 @@
           <t>https://www.premierdevelopment.com/central-nj/luxury-apartments/stone-bridge/</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1271,6 +1306,11 @@
           <t>https://www.premierdevelopment.com/central-nj/luxury-apartments/brookhaven-lofts/</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1363,6 +1403,11 @@
           <t>https://bestrentnj.com/Communities/Rivendell-at-Edison/</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1451,6 +1496,11 @@
           <t>https://www.zillow.com/apartments/watchung-nj/crystal-ridge-at-watchung/5Xj7JZ/</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1539,6 +1589,11 @@
           <t>https://www.liveatthelena.com/floorplans</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1627,6 +1682,11 @@
           <t>https://www.avaloncommunities.com/new-jersey/piscataway-apartments/avalon-piscataway/</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1715,6 +1775,11 @@
           <t>https://www.apartments.com/citizen-bound-brook-bound-brook-nj/39et2kd/</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1803,6 +1868,11 @@
           <t>https://www.theloftsmiddlesex.com/floorplans</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1891,6 +1961,11 @@
           <t>https://www.larkenassociates.com/residential-rentals/hillsborough-village-center</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1979,6 +2054,11 @@
           <t>https://www.premierdevelopment.com/central-nj/luxury-apartments/cedar-manor/</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2067,6 +2147,11 @@
           <t>https://www.apartments.com/sunnymeade-run-hillsborough-nj/2befhwb/</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2155,6 +2240,11 @@
           <t>https://bestrentnj.com/Communities/Pike-Run-Meadows/</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2243,6 +2333,11 @@
           <t>https://bestrentnj.com/Communities/Pike-Run-Village/</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2335,6 +2430,11 @@
           <t>https://bestrentnj.com/Communities/Rivendell-Heights/</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2423,6 +2523,11 @@
           <t>https://bestrentnj.com/Communities/Rivendell-Village/</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2511,6 +2616,11 @@
           <t>https://bestrentnj.com/Communities/Edison-Woods/</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2599,6 +2709,11 @@
           <t>https://bestrentnj.com/Communities/Mae-Brook-at-Renaissance/</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2687,6 +2802,11 @@
           <t>https://bestrentnj.com/Communities/Renaissance-Manor/</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2779,6 +2899,11 @@
           <t>https://bestrentnj.com/Communities/Blueberry-Village/</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2867,6 +2992,11 @@
           <t>https://www.apartments.com/raritan-riverside-raritan-nj/s1kqpf7/</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2955,6 +3085,11 @@
           <t>https://bestrentnj.com/Communities/Amwell-Terrace/</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -3043,6 +3178,11 @@
           <t>https://mi-placehillsborough.com/floor-plans/</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3131,6 +3271,11 @@
           <t>https://www.bluehillnj.com/</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -3215,6 +3360,11 @@
         </is>
       </c>
       <c r="R30" s="4" t="str"/>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -3299,6 +3449,11 @@
         </is>
       </c>
       <c r="R31" s="4" t="str"/>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -3387,6 +3542,11 @@
         </is>
       </c>
       <c r="R32" s="4" t="str"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -3471,6 +3631,11 @@
         </is>
       </c>
       <c r="R33" s="4" t="str"/>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -3555,6 +3720,11 @@
         </is>
       </c>
       <c r="R34" s="4" t="str"/>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -3639,6 +3809,11 @@
         </is>
       </c>
       <c r="R35" s="4" t="str"/>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -3723,6 +3898,11 @@
         </is>
       </c>
       <c r="R36" s="4" t="str"/>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -3807,6 +3987,11 @@
         </is>
       </c>
       <c r="R37" s="4" t="str"/>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -3891,6 +4076,11 @@
         </is>
       </c>
       <c r="R38" s="4" t="str"/>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -3975,6 +4165,11 @@
         </is>
       </c>
       <c r="R39" s="4" t="str"/>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -4059,6 +4254,11 @@
         </is>
       </c>
       <c r="R40" s="4" t="str"/>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -4143,6 +4343,11 @@
         </is>
       </c>
       <c r="R41" s="4" t="str"/>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -4227,6 +4432,11 @@
         </is>
       </c>
       <c r="R42" s="4" t="str"/>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -4311,6 +4521,11 @@
         </is>
       </c>
       <c r="R43" s="4" t="str"/>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -4395,6 +4610,11 @@
         </is>
       </c>
       <c r="R44" s="4" t="str"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -4479,6 +4699,11 @@
         </is>
       </c>
       <c r="R45" s="4" t="str"/>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -4563,6 +4788,11 @@
         </is>
       </c>
       <c r="R46" s="4" t="str"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -4651,6 +4881,11 @@
           <t>https://therockwellgreenbrook.com/</t>
         </is>
       </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -4739,6 +4974,11 @@
           <t>https://www.thekingsleynj.com/</t>
         </is>
       </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -4831,6 +5071,11 @@
           <t>https://bestrentnj.com/Communities/Edison-Lights/</t>
         </is>
       </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -4919,6 +5164,11 @@
           <t>https://bestrentnj.com/Communities/Woodbridge-Center-Plaza/</t>
         </is>
       </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -5007,6 +5257,11 @@
           <t>https://bestrentnj.com/Communities/Woodbridge-Village/</t>
         </is>
       </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -5095,6 +5350,11 @@
           <t>https://bestrentnj.com/Communities/Beekman-Gardens/</t>
         </is>
       </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -5183,6 +5443,11 @@
           <t>https://bestrentnj.com/Communities/The-Glades-at-Beekman/</t>
         </is>
       </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -5271,6 +5536,11 @@
           <t>https://bestrentnj.com/Communities/Boulders-at-Beekman/</t>
         </is>
       </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -5357,6 +5627,11 @@
       <c r="R55" s="4" t="inlineStr">
         <is>
           <t>https://bestrentnj.com/Communities/North-Brunswick-Manor/</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Needs review</t>
         </is>
       </c>
     </row>
@@ -5400,8 +5675,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:S27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -5514,6 +5789,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -5602,6 +5882,11 @@
           <t>https://www.apartments.com/fairway-28-bridgewater-nj/3m3bv0f/</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -5690,6 +5975,11 @@
           <t>https://www.apartments.com/station-house-somerville-nj/0bzvy20/</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -5778,6 +6068,11 @@
           <t>https://www.premierdevelopment.com/central-nj/luxury-apartments/stone-bridge/</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -5866,6 +6161,11 @@
           <t>https://www.apartments.com/raritan-riverside-raritan-nj/s1kqpf7/</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -5954,6 +6254,11 @@
           <t>https://www.liveatthelena.com/floorplans</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -6042,6 +6347,11 @@
           <t>https://www.premierdevelopment.com/central-nj/luxury-apartments/brookhaven-lofts/</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -6130,6 +6440,11 @@
           <t>https://mi-placehillsborough.com/floor-plans/</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -6218,6 +6533,11 @@
           <t>https://bestrentnj.com/Communities/Amwell-Terrace/</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -6306,6 +6626,11 @@
           <t>https://bestrentnj.com/Communities/Pike-Run-Meadows/</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -6394,6 +6719,11 @@
           <t>https://bestrentnj.com/Communities/Pike-Run-Village/</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -6482,6 +6812,11 @@
           <t>https://www.larkenassociates.com/residential-rentals/hillsborough-village-center</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -6570,6 +6905,11 @@
           <t>https://www.apartments.com/sunnymeade-run-hillsborough-nj/2befhwb/</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -6658,6 +6998,11 @@
           <t>https://www.redfin.com/zipcode/08854/2-bedroom-houses-for-rent</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -6746,6 +7091,11 @@
           <t>https://bestrentnj.com/Communities/Edison-Woods/</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -6838,6 +7188,11 @@
           <t>https://bestrentnj.com/Communities/Rivendell-Heights/</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -6926,6 +7281,11 @@
           <t>https://bestrentnj.com/Communities/Rivendell-Village/</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -7014,6 +7374,11 @@
           <t>https://www.avaloncommunities.com/new-jersey/piscataway-apartments/avalon-piscataway/</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -7106,6 +7471,11 @@
           <t>https://bestrentnj.com/Communities/Rivendell-at-Edison/</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -7194,6 +7564,11 @@
           <t>https://www.theloftsmiddlesex.com/floorplans</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -7282,6 +7657,11 @@
           <t>https://www.queensgateapts.com/floorplans</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -7370,6 +7750,11 @@
           <t>https://www.bluehillnj.com/</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -7458,6 +7843,11 @@
           <t>https://www.apartments.com/citizen-bound-brook-bound-brook-nj/39et2kd/</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -7546,6 +7936,11 @@
           <t>https://www.zillow.com/apartments/watchung-nj/crystal-ridge-at-watchung/5Xj7JZ/</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -7634,6 +8029,11 @@
           <t>https://www.premierdevelopment.com/central-nj/luxury-apartments/cedar-manor/</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -7722,6 +8122,11 @@
           <t>https://bestrentnj.com/Communities/Mae-Brook-at-Renaissance/</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -7808,6 +8213,11 @@
       <c r="R27" s="4" t="inlineStr">
         <is>
           <t>https://bestrentnj.com/Communities/Renaissance-Manor/</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Needs review</t>
         </is>
       </c>
     </row>
@@ -7834,8 +8244,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
@@ -7855,6 +8265,11 @@
       <c r="F1" s="1" t="n"/>
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
     </row>
     <row r="2"/>
     <row r="3">
@@ -7898,6 +8313,11 @@
           <t>Suggested combined tour</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -7940,6 +8360,11 @@
           <t>Bridgewater + Raritan + Somerville</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -7982,6 +8407,11 @@
           <t>Hillsborough + Belle Mead</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -8024,6 +8454,11 @@
           <t>Edison + Piscataway + Middlesex/Dunellen + South Plainfield</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -8066,6 +8501,11 @@
           <t>Bound Brook + South Bound Brook + Watchung + Green Brook</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -8108,6 +8548,11 @@
           <t>Somerset + Franklin Park</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
@@ -8145,6 +8590,11 @@
           <t>New/North Brunswick + South Brunswick/Monmouth Junction</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
@@ -8182,6 +8632,11 @@
           <t>Woodbridge + Avenel</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="45" t="inlineStr">
@@ -8224,6 +8679,11 @@
           <t>Count</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8266,6 +8726,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8308,6 +8773,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8350,6 +8820,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8392,6 +8867,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8434,6 +8914,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8474,6 +8959,11 @@
       <c r="H17" t="inlineStr">
         <is>
           <t>27</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Needs review</t>
         </is>
       </c>
     </row>
@@ -8492,6 +8982,11 @@
       <c r="F20" s="1" t="n"/>
       <c r="G20" s="1" t="n"/>
       <c r="H20" s="1" t="n"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>